<commit_message>
Correct some small mistakes for adding PLAN-DB schema
</commit_message>
<xml_diff>
--- a/ckanext/lhm/schemas/template_master.xlsx
+++ b/ckanext/lhm/schemas/template_master.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\home\mb\p2\ckanext-lhm\ckanext\lhm\schemas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04323879-7628-4EC9-9E0A-80199A761134}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5E13F00-D7CC-45C3-806A-7A8B48DF3D54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="871" xr2:uid="{EFAD0BDA-2C19-4F99-80E8-84599936D919}"/>
   </bookViews>
@@ -797,15 +797,9 @@
     <t>PLAN_MD_update-zyklus</t>
   </si>
   <si>
-    <t>quartalsweise</t>
-  </si>
-  <si>
     <t>Jährlich</t>
   </si>
   <si>
-    <t>zweijährlich</t>
-  </si>
-  <si>
     <t>PLAN_MD_schema</t>
   </si>
   <si>
@@ -864,6 +858,12 @@
   </si>
   <si>
     <t>ZEN</t>
+  </si>
+  <si>
+    <t>Quartalsweise</t>
+  </si>
+  <si>
+    <t>Zweijährlich</t>
   </si>
 </sst>
 </file>
@@ -2370,7 +2370,7 @@
         <v>229</v>
       </c>
       <c r="W1" s="5" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="X1" s="5" t="s">
         <v>243</v>
@@ -2440,7 +2440,7 @@
         <v>230</v>
       </c>
       <c r="W2" s="3" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="X2" s="2" t="s">
         <v>104</v>
@@ -2514,7 +2514,7 @@
         <v>231</v>
       </c>
       <c r="W3" s="3" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="X3" s="2" t="s">
         <v>143</v>
@@ -2579,7 +2579,7 @@
         <v>242</v>
       </c>
       <c r="W4" s="3" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="X4" s="2" t="s">
         <v>144</v>
@@ -2623,7 +2623,7 @@
         <v>90</v>
       </c>
       <c r="W5" s="3" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="X5" s="2" t="s">
         <v>145</v>
@@ -2667,7 +2667,7 @@
         <v>195</v>
       </c>
       <c r="W6" s="3" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="X6" s="2" t="s">
         <v>146</v>
@@ -2705,7 +2705,7 @@
         <v>194</v>
       </c>
       <c r="W7" s="3" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="X7" s="2" t="s">
         <v>105</v>
@@ -2743,10 +2743,10 @@
         <v>196</v>
       </c>
       <c r="W8" s="3" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="X8" s="2" t="s">
-        <v>244</v>
+        <v>265</v>
       </c>
     </row>
     <row r="9" spans="1:24">
@@ -2770,10 +2770,10 @@
         <v>198</v>
       </c>
       <c r="W9" s="3" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="X9" s="2" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="10" spans="1:24">
@@ -2798,10 +2798,10 @@
         <v>197</v>
       </c>
       <c r="W10" s="3" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="X10" s="2" t="s">
-        <v>246</v>
+        <v>266</v>
       </c>
     </row>
     <row r="11" spans="1:24">
@@ -2826,7 +2826,7 @@
         <v>199</v>
       </c>
       <c r="W11" s="3" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="X11" s="2" t="s">
         <v>106</v>
@@ -2848,7 +2848,7 @@
         <v>200</v>
       </c>
       <c r="W12" s="3" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
     </row>
     <row r="13" spans="1:24">
@@ -2864,7 +2864,7 @@
       <c r="E13" s="1"/>
       <c r="K13" s="15"/>
       <c r="W13" s="3" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
     </row>
     <row r="14" spans="1:24">
@@ -2880,7 +2880,7 @@
       <c r="E14" s="1"/>
       <c r="K14" s="15"/>
       <c r="W14" s="3" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
     </row>
     <row r="15" spans="1:24">
@@ -2896,7 +2896,7 @@
       <c r="E15" s="1"/>
       <c r="K15" s="15"/>
       <c r="W15" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="16" spans="1:24">
@@ -2912,7 +2912,7 @@
       <c r="E16" s="1"/>
       <c r="K16" s="15"/>
       <c r="W16" s="3" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="17" spans="1:23">
@@ -2928,7 +2928,7 @@
       <c r="E17" s="1"/>
       <c r="K17" s="15"/>
       <c r="W17" s="3" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
     </row>
     <row r="18" spans="1:23">
@@ -2960,7 +2960,7 @@
       <c r="E19" s="1"/>
       <c r="K19" s="15"/>
       <c r="W19" s="3" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
     </row>
     <row r="20" spans="1:23">
@@ -2976,7 +2976,7 @@
       <c r="E20" s="1"/>
       <c r="K20" s="15"/>
       <c r="W20" s="3" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
     </row>
     <row r="21" spans="1:23">
@@ -2992,7 +2992,7 @@
       <c r="E21" s="1"/>
       <c r="K21" s="15"/>
       <c r="W21" s="3" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
     </row>
     <row r="22" spans="1:23">
@@ -3087,7 +3087,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="PH4zrp7eXCCYTe30bZgWa4oN323isiTnw119OHfSlXEE4aKSPiWff8viQcR9grAl1yuVHM8VUpNSbGDq2VjIJA==" saltValue="JZVoZuV7oNQazjtxqkPBpg==" spinCount="100000" sheet="1" formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="XIhFgadR1bmyL3SPoHS41+3tUZqsLtqcbU4VzMIUMew96ptGIJKwvbDRU4h465yFQ0fDb5h+uNZvr6erUHABag==" saltValue="nyUB6A+Q9PWi/8oZYGFrAA==" spinCount="100000" sheet="1" formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>